<commit_message>
docs: add further verified QRL papers
</commit_message>
<xml_diff>
--- a/metadata/QRL.xlsx
+++ b/metadata/QRL.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R42969e183f374649"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R8526255881ac4ec4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -959,19 +959,19 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" t="str">
-        <x:v>Qtrl: Toward practical quantum reinforcement learning via quantum-train</x:v>
+        <x:v>Auxiliary Task-Based Deep Reinforcement Learning for Quantum Control</x:v>
       </x:c>
       <x:c r="B33" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="C33" t="str">
-        <x:v>arXiv</x:v>
+        <x:v>IEEE</x:v>
       </x:c>
       <x:c r="D33" t="str">
-        <x:v>Liu, Chen-Yu, et al.</x:v>
+        <x:v>Shumin Zhou; Hailan Ma; Sen Kuang; Daoyi Dong</x:v>
       </x:c>
       <x:c r="E33" t="str">
-        <x:v>https://arxiv.org/pdf/2407.06103</x:v>
+        <x:v>https://doi.org/10.1109/TCYB.2024.3521300</x:v>
       </x:c>
       <x:c r="F33" t="str">
         <x:v>QRL</x:v>
@@ -979,19 +979,19 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" t="str">
-        <x:v>Hybrid actor-critic algorithm for quantum reinforcement learning at CERN beam lines</x:v>
+        <x:v>Robust quantum control using reinforcement learning from demonstration</x:v>
       </x:c>
       <x:c r="B34" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="C34" t="str">
-        <x:v>Quantum Science and Technology </x:v>
+        <x:v>Nature</x:v>
       </x:c>
       <x:c r="D34" t="str">
-        <x:v>Schenk, Michael, et al.</x:v>
+        <x:v>Shengyong Li; Yidian Fan; Xiang Li; Xinhui Ruan; Qianchuan Zhao; Zhihui Peng; Re-Bing Wu; Jing Zhang; Pengtao Song</x:v>
       </x:c>
       <x:c r="E34" t="str">
-        <x:v>https://iopscience.iop.org/article/10.1088/2058-9565/ad261b/meta</x:v>
+        <x:v>https://doi.org/10.1038/s41534-025-01065-2</x:v>
       </x:c>
       <x:c r="F34" t="str">
         <x:v>QRL</x:v>
@@ -999,19 +999,19 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" t="str">
-        <x:v>Differentiable Quantum Architecture Search in Asynchronous Quantum Reinforcement Learning.</x:v>
+        <x:v>Hybrid quantum-classical reinforcement learning in latent observation spaces</x:v>
       </x:c>
       <x:c r="B35" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="C35" t="str">
-        <x:v>arXiv</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D35" t="str">
-        <x:v>Chen, Samuel Yen-Chi.</x:v>
+        <x:v>Dániel T. R. Nagy; Csaba Czabán; Bence Bakó; Péter Hága; Zsófia Kallus; Zoltán Zimborás</x:v>
       </x:c>
       <x:c r="E35" t="str">
-        <x:v>https://arxiv.org/pdf/2407.18202</x:v>
+        <x:v>https://doi.org/10.1007/s42484-025-00306-z</x:v>
       </x:c>
       <x:c r="F35" t="str">
         <x:v>QRL</x:v>
@@ -1019,776 +1019,776 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" t="str">
+        <x:v>Reinforcement Learning to Learn Quantum States for Heisenberg Scaling Accuracy</x:v>
+      </x:c>
+      <x:c r="B36" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C36" t="str">
+        <x:v>Wiley</x:v>
+      </x:c>
+      <x:c r="D36" t="str">
+        <x:v>Jeongwoo Jae; J. Hong; J. Choo; Young-Duk Kwon</x:v>
+      </x:c>
+      <x:c r="E36" t="str">
+        <x:v>https://doi.org/10.1002/qute.202500206</x:v>
+      </x:c>
+      <x:c r="F36" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>Toward Heisenberg Limit without Critical Slowing Down via Quantum Reinforcement Learning</x:v>
+      </x:c>
+      <x:c r="B37" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>APS</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>Hang Xu; Tailong Xiao; Jingzheng Huang; Ming He; Jianping Fan; Guihua Zeng</x:v>
+      </x:c>
+      <x:c r="E37" t="str">
+        <x:v>https://doi.org/10.1103/PhysRevLett.134.120803</x:v>
+      </x:c>
+      <x:c r="F37" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>Quantum reinforcement learning in continuous action space</x:v>
+      </x:c>
+      <x:c r="B38" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C38" t="str">
+        <x:v>Quantum</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
+        <x:v>Shaojun Wu; Shan Jin; Dingding Wen; Donghong Han; Xiaoting Wang</x:v>
+      </x:c>
+      <x:c r="E38" t="str">
+        <x:v>https://doi.org/10.22331/q-2025-03-12-1660</x:v>
+      </x:c>
+      <x:c r="F38" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" t="str">
+        <x:v>Nav-Q: quantum deep reinforcement learning for collision-free navigation of self-driving cars</x:v>
+      </x:c>
+      <x:c r="B39" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C39" t="str">
+        <x:v>Springer</x:v>
+      </x:c>
+      <x:c r="D39" t="str">
+        <x:v>Akash Sinha; Antonio Macaluso; Matthias Klusch</x:v>
+      </x:c>
+      <x:c r="E39" t="str">
+        <x:v>https://doi.org/10.1007/s42484-024-00226-4</x:v>
+      </x:c>
+      <x:c r="F39" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" t="str">
+        <x:v>A hybrid learning agent for episodic learning tasks with unknown target distance</x:v>
+      </x:c>
+      <x:c r="B40" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C40" t="str">
+        <x:v>Springer</x:v>
+      </x:c>
+      <x:c r="D40" t="str">
+        <x:v>Oliver Sefrin; Sabine Wölk</x:v>
+      </x:c>
+      <x:c r="E40" t="str">
+        <x:v>https://doi.org/10.1007/s42484-025-00269-1</x:v>
+      </x:c>
+      <x:c r="F40" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" t="str">
+        <x:v>Qtrl: Toward practical quantum reinforcement learning via quantum-train</x:v>
+      </x:c>
+      <x:c r="B41" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C41" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D41" t="str">
+        <x:v>Liu, Chen-Yu, et al.</x:v>
+      </x:c>
+      <x:c r="E41" t="str">
+        <x:v>https://arxiv.org/pdf/2407.06103</x:v>
+      </x:c>
+      <x:c r="F41" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="str">
+        <x:v>Hybrid actor-critic algorithm for quantum reinforcement learning at CERN beam lines</x:v>
+      </x:c>
+      <x:c r="B42" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C42" t="str">
+        <x:v>Quantum Science and Technology </x:v>
+      </x:c>
+      <x:c r="D42" t="str">
+        <x:v>Schenk, Michael, et al.</x:v>
+      </x:c>
+      <x:c r="E42" t="str">
+        <x:v>https://iopscience.iop.org/article/10.1088/2058-9565/ad261b/meta</x:v>
+      </x:c>
+      <x:c r="F42" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" t="str">
+        <x:v>Differentiable Quantum Architecture Search in Asynchronous Quantum Reinforcement Learning.</x:v>
+      </x:c>
+      <x:c r="B43" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C43" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D43" t="str">
+        <x:v>Chen, Samuel Yen-Chi.</x:v>
+      </x:c>
+      <x:c r="E43" t="str">
+        <x:v>https://arxiv.org/pdf/2407.18202</x:v>
+      </x:c>
+      <x:c r="F43" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
         <x:v>Quantum Reinforcement Learning for Spatio-Temporal Prioritization in Metaverse
 </x:v>
       </x:c>
-      <x:c r="B36" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C36" t="str">
+      <x:c r="B44" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
         <x:v>IEEE Access</x:v>
       </x:c>
-      <x:c r="D36" t="str">
+      <x:c r="D44" t="str">
         <x:v>Park, Soohyun, Hankyul Baek, and Joongheon Kim.</x:v>
       </x:c>
-      <x:c r="E36" t="str">
+      <x:c r="E44" t="str">
         <x:v>https://ieeexplore.ieee.org/document/10501929?denied=</x:v>
       </x:c>
-      <x:c r="F36" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" t="str">
+      <x:c r="F44" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="str">
         <x:v>Brain-Inspired Agents for Quantum Reinforcement Learning
 </x:v>
       </x:c>
-      <x:c r="B37" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C37" t="str">
+      <x:c r="B45" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C45" t="str">
         <x:v>Mathematics</x:v>
       </x:c>
-      <x:c r="D37" t="str">
+      <x:c r="D45" t="str">
         <x:v>Andrés, Eva, Manuel Pegalajar Cuéllar, and Gabriel Navarro.</x:v>
       </x:c>
-      <x:c r="E37" t="str">
+      <x:c r="E45" t="str">
         <x:v>https://www.mdpi.com/2227-7390/12/8/1230</x:v>
       </x:c>
-      <x:c r="F37" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38">
-      <x:c r="A38" t="str">
+      <x:c r="F45" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="str">
         <x:v>Realizing Stabilized Landing for Computation-Limited Reusable Rockets: A Quantum Reinforcement Learning Approach</x:v>
       </x:c>
-      <x:c r="B38" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C38" t="str">
+      <x:c r="B46" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C46" t="str">
         <x:v>IEEE Transactions on Vehicular Technology</x:v>
       </x:c>
-      <x:c r="D38" t="str">
+      <x:c r="D46" t="str">
         <x:v>Kim, Gyu Seon, Jaehyun Chung, and Soohyun Park.</x:v>
       </x:c>
-      <x:c r="E38" t="str">
+      <x:c r="E46" t="str">
         <x:v>https://ieeexplore.ieee.org/abstract/document/10461080</x:v>
       </x:c>
-      <x:c r="F38" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" t="str">
+      <x:c r="F46" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" t="str">
         <x:v>Efficient relation extraction via quantum reinforcement learning</x:v>
       </x:c>
-      <x:c r="B39" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C39" t="str">
+      <x:c r="B47" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C47" t="str">
         <x:v>Complex &amp; Intelligent Systems </x:v>
       </x:c>
-      <x:c r="D39" t="str">
+      <x:c r="D47" t="str">
         <x:v>Zhu, Xianchao, et al.</x:v>
       </x:c>
-      <x:c r="E39" t="str">
+      <x:c r="E47" t="str">
         <x:v>https://link.springer.com/article/10.1007/s40747-024-01381-8</x:v>
       </x:c>
-      <x:c r="F39" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" t="str">
+      <x:c r="F47" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
         <x:v>Hamiltonian-based Quantum Reinforcement Learning for Neural Combinatorial Optimization.</x:v>
       </x:c>
-      <x:c r="B40" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C40" t="str">
+      <x:c r="B48" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D40" t="str">
+      <x:c r="D48" t="str">
         <x:v>Kruse, Georg, et al.</x:v>
       </x:c>
-      <x:c r="E40" t="str">
+      <x:c r="E48" t="str">
         <x:v>https://arxiv.org/pdf/2405.07790</x:v>
       </x:c>
-      <x:c r="F40" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" t="str">
+      <x:c r="F48" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
         <x:v>Hype or Heuristic? Quantum Reinforcement Learning for Join Order Optimisation.</x:v>
       </x:c>
-      <x:c r="B41" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C41" t="str">
+      <x:c r="B49" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D41" t="str">
+      <x:c r="D49" t="str">
         <x:v>Franz, Maja, et al.</x:v>
       </x:c>
-      <x:c r="E41" t="str">
+      <x:c r="E49" t="str">
         <x:v>https://arxiv.org/pdf/2405.07770</x:v>
       </x:c>
-      <x:c r="F41" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42" t="str">
+      <x:c r="F49" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
         <x:v>Automatic evolutionary design of quantum rule-based systems and applications to quantum reinforcement learning</x:v>
       </x:c>
-      <x:c r="B42" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C42" t="str">
+      <x:c r="B50" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
         <x:v>Quantum Information Processing</x:v>
       </x:c>
-      <x:c r="D42" t="str">
+      <x:c r="D50" t="str">
         <x:v>Cuéllar, Manuel P., M. C. Pegalajar, and C. Cano.</x:v>
       </x:c>
-      <x:c r="E42" t="str">
+      <x:c r="E50" t="str">
         <x:v>https://link.springer.com/article/10.1007/s11128-024-04391-0</x:v>
       </x:c>
-      <x:c r="F42" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" t="str">
+      <x:c r="F50" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
         <x:v>Efficient Quantum Recurrent Reinforcement Learning Via Quantum Reservoir Computing
 </x:v>
       </x:c>
-      <x:c r="B43" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C43" t="str">
+      <x:c r="B51" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
         <x:v>IEEE International Conference on Acoustics, Speech and Signal Processing (ICASSP)</x:v>
       </x:c>
-      <x:c r="D43" t="str">
+      <x:c r="D51" t="str">
         <x:v>Chen, Samuel Yen-Chi.</x:v>
       </x:c>
-      <x:c r="E43" t="str">
+      <x:c r="E51" t="str">
         <x:v>https://ieeexplore.ieee.org/abstract/document/10446089</x:v>
       </x:c>
-      <x:c r="F43" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44">
-      <x:c r="A44" t="str">
+      <x:c r="F51" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
         <x:v>Quafu-RL: The cloud quantum computers based quantum reinforcement learning
 </x:v>
       </x:c>
-      <x:c r="B44" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C44" t="str">
+      <x:c r="B52" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
         <x:v>Chinese Physics </x:v>
       </x:c>
-      <x:c r="D44" t="str">
+      <x:c r="D52" t="str">
         <x:v>Jin, Yu-Xin, et al.</x:v>
       </x:c>
-      <x:c r="E44" t="str">
+      <x:c r="E52" t="str">
         <x:v>https://iopscience.iop.org/article/10.1088/1674-1056/ad3061/meta</x:v>
       </x:c>
-      <x:c r="F44" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45">
-      <x:c r="A45" t="str">
+      <x:c r="F52" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
         <x:v>Quantum Advantage Actor-Critic for Reinforcement Learning
 </x:v>
       </x:c>
-      <x:c r="B45" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C45" t="str">
+      <x:c r="B53" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D45" t="str">
+      <x:c r="D53" t="str">
         <x:v>Kölle, Michael, et al.</x:v>
       </x:c>
-      <x:c r="E45" t="str">
+      <x:c r="E53" t="str">
         <x:v>https://arxiv.org/abs/2401.07043</x:v>
       </x:c>
-      <x:c r="F45" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46" t="str">
+      <x:c r="F53" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
         <x:v>Joint Quantum Reinforcement Learning and Stabilized Control for Spatio-Temporal Coordination in Metaverse</x:v>
       </x:c>
-      <x:c r="B46" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C46" t="str">
+      <x:c r="B54" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
         <x:v>IEEE Transactions on Mobile Computing</x:v>
       </x:c>
-      <x:c r="D46" t="str">
+      <x:c r="D54" t="str">
         <x:v>Park, Soohyun, et al.</x:v>
       </x:c>
-      <x:c r="E46" t="str">
+      <x:c r="E54" t="str">
         <x:v>https://ieeexplore.ieee.org/abstract/document/10543150</x:v>
       </x:c>
-      <x:c r="F46" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47">
-      <x:c r="A47" t="str">
+      <x:c r="F54" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" t="str">
         <x:v>Reinforcement learning assisted recursive QAOA
 </x:v>
       </x:c>
-      <x:c r="B47" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C47" t="str">
+      <x:c r="B55" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C55" t="str">
         <x:v>EPJ Quantum Technology </x:v>
       </x:c>
-      <x:c r="D47" t="str">
+      <x:c r="D55" t="str">
         <x:v>Patel, Yash J., et al.</x:v>
       </x:c>
-      <x:c r="E47" t="str">
+      <x:c r="E55" t="str">
         <x:v>https://epjqt.epj.org/articles/epjqt/abs/2024/01/40507_2023_Article_214/40507_2023_Article_214.html</x:v>
       </x:c>
-      <x:c r="F47" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48">
-      <x:c r="A48" t="str">
+      <x:c r="F55" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" t="str">
         <x:v>A Study on Optimization Techniques for Variational Quantum Circuits in Reinforcement Learning
 </x:v>
       </x:c>
-      <x:c r="B48" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C48" t="str">
+      <x:c r="B56" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C56" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D48" t="str">
+      <x:c r="D56" t="str">
         <x:v>Kölle, Michael, et al.</x:v>
       </x:c>
-      <x:c r="E48" t="str">
+      <x:c r="E56" t="str">
         <x:v>https://arxiv.org/abs/2405.12354</x:v>
       </x:c>
-      <x:c r="F48" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" t="str">
+      <x:c r="F56" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" t="str">
         <x:v>eQMARL: Entangled Quantum Multi-Agent Reinforcement Learning for Distributed Cooperation over Quantum Channels
 </x:v>
       </x:c>
-      <x:c r="B49" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C49" t="str">
+      <x:c r="B57" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C57" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D49" t="str">
+      <x:c r="D57" t="str">
         <x:v>DeRieux, Alexander, and Walid Saad.</x:v>
       </x:c>
-      <x:c r="E49" t="str">
+      <x:c r="E57" t="str">
         <x:v>https://arxiv.org/abs/2405.17486</x:v>
       </x:c>
-      <x:c r="F49" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="50">
-      <x:c r="A50" t="str">
+      <x:c r="F57" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" t="str">
         <x:v>Quantum Reinforcement Learning in Non-Abelian Environments: Unveiling Novel Formulations and Quantum Advantage Exploration</x:v>
       </x:c>
-      <x:c r="B50" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C50" t="str">
+      <x:c r="B58" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C58" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D50" t="str">
+      <x:c r="D58" t="str">
         <x:v>Ghosal, Shubhayan.</x:v>
       </x:c>
-      <x:c r="E50" t="str">
+      <x:c r="E58" t="str">
         <x:v>https://arxiv.org/abs/2406.06531</x:v>
       </x:c>
-      <x:c r="F50" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="51">
-      <x:c r="A51" t="str">
+      <x:c r="F58" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" t="str">
         <x:v>Reinforcement Learning for Variational Quantum Circuits Design
 </x:v>
       </x:c>
-      <x:c r="B51" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C51" t="str">
+      <x:c r="B59" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C59" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D51" t="str">
+      <x:c r="D59" t="str">
         <x:v>Foderà, Simone, et al.</x:v>
       </x:c>
-      <x:c r="E51" t="str">
+      <x:c r="E59" t="str">
         <x:v>https://arxiv.org/abs/2409.05475</x:v>
       </x:c>
-      <x:c r="F51" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="52">
-      <x:c r="A52" t="str">
+      <x:c r="F59" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" t="str">
         <x:v>CURRICULUM REINFORCEMENT LEARNING FOR
 QUANTUM ARCHITECTURE SEARCH UNDER HARDWARE ERROR</x:v>
       </x:c>
-      <x:c r="B52" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C52" t="str">
+      <x:c r="B60" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C60" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D52"/>
-      <x:c r="E52" t="str">
+      <x:c r="D60"/>
+      <x:c r="E60" t="str">
         <x:v>https://arxiv.org/pdf/2402.03500</x:v>
       </x:c>
-      <x:c r="F52" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="53">
-      <x:c r="A53" t="str">
+      <x:c r="F60" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="str">
         <x:v>Fast and reliable entanglement distribution with quantum repeaters: Principles for improving protocols using reinforcement learning</x:v>
       </x:c>
-      <x:c r="B53" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C53" t="str">
+      <x:c r="B61" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C61" t="str">
         <x:v>Physical Review Applied </x:v>
       </x:c>
-      <x:c r="D53" t="str">
+      <x:c r="D61" t="str">
         <x:v>Haldar, Stav, et al.</x:v>
       </x:c>
-      <x:c r="E53" t="str">
+      <x:c r="E61" t="str">
         <x:v>https://journals.aps.org/prapplied/abstract/10.1103/PhysRevApplied.21.024041</x:v>
       </x:c>
-      <x:c r="F53" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="54">
-      <x:c r="A54" t="str">
+      <x:c r="F61" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" t="str">
         <x:v>A Reinforcement Learning Environment for Directed Quantum Circuit Synthesis
 </x:v>
       </x:c>
-      <x:c r="B54" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C54" t="str">
+      <x:c r="B62" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C62" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D54" t="str">
+      <x:c r="D62" t="str">
         <x:v>Kölle, Michael, et al.</x:v>
       </x:c>
-      <x:c r="E54" t="str">
+      <x:c r="E62" t="str">
         <x:v>https://arxiv.org/abs/2401.07054</x:v>
       </x:c>
-      <x:c r="F54" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55">
-      <x:c r="A55" t="str">
+      <x:c r="F62" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" t="str">
         <x:v>Arbitrary quantum states preparation aided by deep reinforcement learning
 </x:v>
       </x:c>
-      <x:c r="B55" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C55" t="str">
+      <x:c r="B63" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C63" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D55" t="str">
+      <x:c r="D63" t="str">
         <x:v>Wang, Zhao-Wei, and Zhao-Ming Wang.</x:v>
       </x:c>
-      <x:c r="E55" t="str">
+      <x:c r="E63" t="str">
         <x:v>https://arxiv.org/abs/2407.16368</x:v>
       </x:c>
-      <x:c r="F55" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56">
-      <x:c r="A56" t="str">
+      <x:c r="F63" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" t="str">
         <x:v>Principles of Quantum Reinforcement Learning
 </x:v>
       </x:c>
-      <x:c r="B56" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C56" t="str">
+      <x:c r="B64" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C64" t="str">
         <x:v>Data Science And Engineering</x:v>
       </x:c>
-      <x:c r="D56" t="str">
+      <x:c r="D64" t="str">
         <x:v>Pacifico, Michele. Principles of Quantum Reinforcement Learning. Diss. Politecnico di Torino, 2024.</x:v>
       </x:c>
-      <x:c r="E56" t="str">
+      <x:c r="E64" t="str">
         <x:v>https://webthesis.biblio.polito.it/30877/</x:v>
       </x:c>
-      <x:c r="F56" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="57">
-      <x:c r="A57" t="str">
+      <x:c r="F64" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" t="str">
         <x:v>Applications of model-aware reinforcement learning in Bayesian quantum metrology</x:v>
       </x:c>
-      <x:c r="B57" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C57" t="str">
+      <x:c r="B65" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C65" t="str">
         <x:v>Physical Review A </x:v>
       </x:c>
-      <x:c r="D57" t="str">
+      <x:c r="D65" t="str">
         <x:v>Belliardo, Federico, Fabio Zoratti, and Vittorio Giovannetti.</x:v>
       </x:c>
-      <x:c r="E57" t="str">
+      <x:c r="E65" t="str">
         <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.109.062609</x:v>
       </x:c>
-      <x:c r="F57" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="58">
-      <x:c r="A58" t="str">
+      <x:c r="F65" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" t="str">
         <x:v>Enhancing variational quantum state diagonalization using reinforcement learning techniques
 </x:v>
       </x:c>
-      <x:c r="B58" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C58" t="str">
+      <x:c r="B66" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C66" t="str">
         <x:v>New Journal of Physics</x:v>
       </x:c>
-      <x:c r="D58" t="str">
+      <x:c r="D66" t="str">
         <x:v>Kundu, Akash, et al.</x:v>
       </x:c>
-      <x:c r="E58" t="str">
+      <x:c r="E66" t="str">
         <x:v>https://iopscience.iop.org/article/10.1088/1367-2630/ad1b7f/meta</x:v>
       </x:c>
-      <x:c r="F58" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="59">
-      <x:c r="A59" t="str">
+      <x:c r="F66" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" t="str">
         <x:v>Quantum Multi-Agent Reinforcement Learning for Aerial Ad-hoc Networks
 </x:v>
       </x:c>
-      <x:c r="B59" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C59" t="str">
+      <x:c r="B67" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C67" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D59" t="str">
+      <x:c r="D67" t="str">
         <x:v>Drăgan, Theodora-Augustina, et al.</x:v>
       </x:c>
-      <x:c r="E59" t="str">
+      <x:c r="E67" t="str">
         <x:v>https://arxiv.org/abs/2404.17499</x:v>
       </x:c>
-      <x:c r="F59" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="60">
-      <x:c r="A60" t="str">
+      <x:c r="F67" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" t="str">
         <x:v>Reinforcement learning-assisted quantum architecture search for variational quantum algorithms
 </x:v>
       </x:c>
-      <x:c r="B60" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C60" t="str">
+      <x:c r="B68" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C68" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D60" t="str">
+      <x:c r="D68" t="str">
         <x:v>Kundu, Akash.</x:v>
       </x:c>
-      <x:c r="E60" t="str">
+      <x:c r="E68" t="str">
         <x:v>https://arxiv.org/abs/2402.13754</x:v>
       </x:c>
-      <x:c r="F60" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="61">
-      <x:c r="A61" t="str">
+      <x:c r="F68" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" t="str">
         <x:v>Design and Analysis of Quantum Transfer Fractal Priority Replay and Mirdad Priority Loss Algorithms for Quantum Reinforcement Learning</x:v>
       </x:c>
-      <x:c r="B61" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C61" t="str">
+      <x:c r="B69" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C69" t="str">
         <x:v>International Conference on Data Management, Analytics &amp; Innovation. Singapore: Springer Nature Singapore</x:v>
       </x:c>
-      <x:c r="D61" t="str">
+      <x:c r="D69" t="str">
         <x:v>Palanivel, R., and P. Muthulakshmi.</x:v>
       </x:c>
-      <x:c r="E61" t="str">
+      <x:c r="E69" t="str">
         <x:v>https://link.springer.com/chapter/10.1007/978-981-97-3242-5_27</x:v>
       </x:c>
-      <x:c r="F61" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="62">
-      <x:c r="A62" t="str">
+      <x:c r="F69" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="str">
         <x:v>Quantum Machine Learning Architecture Search via Deep Reinforcement Learning
 </x:v>
       </x:c>
-      <x:c r="B62" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C62" t="str">
+      <x:c r="B70" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C70" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D62" t="str">
+      <x:c r="D70" t="str">
         <x:v>Dai, Xin, et al.</x:v>
       </x:c>
-      <x:c r="E62" t="str">
+      <x:c r="E70" t="str">
         <x:v>https://arxiv.org/pdf/2407.20147</x:v>
       </x:c>
-      <x:c r="F62" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="63">
-      <x:c r="A63" t="str">
+      <x:c r="F70" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
         <x:v>Model-based Offline Quantum Reinforcement Learning
 </x:v>
       </x:c>
-      <x:c r="B63" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C63" t="str">
+      <x:c r="B71" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C71" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D63" t="str">
+      <x:c r="D71" t="str">
         <x:v>Eisenmann, Simon, et al.</x:v>
       </x:c>
-      <x:c r="E63" t="str">
+      <x:c r="E71" t="str">
         <x:v>https://arxiv.org/abs/2404.10017</x:v>
       </x:c>
-      <x:c r="F63" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="64">
-      <x:c r="A64" t="str">
+      <x:c r="F71" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
         <x:v>A generic and robust quantum agent inspired by deep meta-reinforcement learning</x:v>
       </x:c>
-      <x:c r="B64" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C64" t="str">
+      <x:c r="B72" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="D64" t="str">
+      <x:c r="D72" t="str">
         <x:v>Miao, Zibo, et al.</x:v>
       </x:c>
-      <x:c r="E64" t="str">
+      <x:c r="E72" t="str">
         <x:v>https://arxiv.org/abs/2406.07225</x:v>
       </x:c>
-      <x:c r="F64" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="65">
-      <x:c r="A65" t="str">
+      <x:c r="F72" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="str">
         <x:v>Quantum Entropy and Reinforcement Learning for Distributed Denial of Service Attack Detection in Smart Grid
 </x:v>
       </x:c>
-      <x:c r="B65" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C65" t="str">
+      <x:c r="B73" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C73" t="str">
         <x:v>IEEE Access </x:v>
       </x:c>
-      <x:c r="D65" t="str">
+      <x:c r="D73" t="str">
         <x:v>Said, Dhaou, et al.</x:v>
       </x:c>
-      <x:c r="E65" t="str">
+      <x:c r="E73" t="str">
         <x:v>https://ieeexplore.ieee.org/abstract/document/10633715</x:v>
-      </x:c>
-      <x:c r="F65" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="66">
-      <x:c r="A66" t="str">
-        <x:v>Reinforcement learning-based architecture search for quantum machine learning</x:v>
-      </x:c>
-      <x:c r="B66" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C66" t="str">
-        <x:v>arXiv</x:v>
-      </x:c>
-      <x:c r="D66" t="str">
-        <x:v>Rapp, Frederic, David A. Kreplin, and Marco Roth.</x:v>
-      </x:c>
-      <x:c r="E66" t="str">
-        <x:v>https://arxiv.org/abs/2406.02717</x:v>
-      </x:c>
-      <x:c r="F66" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="67">
-      <x:c r="A67" t="str">
-        <x:v>Attention-Based Deep Reinforcement Learning for Qubit Allocation in Modular Quantum Architectures.</x:v>
-      </x:c>
-      <x:c r="B67" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C67" t="str">
-        <x:v>arXiv</x:v>
-      </x:c>
-      <x:c r="D67" t="str">
-        <x:v>Russo, Enrico, et al.</x:v>
-      </x:c>
-      <x:c r="E67" t="str">
-        <x:v>https://arxiv.org/abs/2406.11452</x:v>
-      </x:c>
-      <x:c r="F67" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="68">
-      <x:c r="A68" t="str">
-        <x:v>Quantum reinforcement learning via policy iteration</x:v>
-      </x:c>
-      <x:c r="B68" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C68" t="str">
-        <x:v>Springer</x:v>
-      </x:c>
-      <x:c r="D68" t="str">
-        <x:v>El Amine Cherrat, Iordanis Kerenidis, Anupam Prakash </x:v>
-      </x:c>
-      <x:c r="E68" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00116-1</x:v>
-      </x:c>
-      <x:c r="F68" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="69">
-      <x:c r="A69" t="str">
-        <x:v>Policy gradients using variational quantum circuits</x:v>
-      </x:c>
-      <x:c r="B69" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C69" t="str">
-        <x:v>Springer</x:v>
-      </x:c>
-      <x:c r="D69" t="str">
-        <x:v>André Sequeira, Luis Paulo Santos, Luis Soares Barbosa </x:v>
-      </x:c>
-      <x:c r="E69" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00101-8</x:v>
-      </x:c>
-      <x:c r="F69" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="70">
-      <x:c r="A70" t="str">
-        <x:v>Robustness of quantum reinforcement learning under hardware errors</x:v>
-      </x:c>
-      <x:c r="B70" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C70" t="str">
-        <x:v>Springer</x:v>
-      </x:c>
-      <x:c r="D70" t="str">
-        <x:v>Andrea Skolik, Stefano Mangini, Thomas Bäck, Chiara Macchiavello &amp; Vedran Dunjko </x:v>
-      </x:c>
-      <x:c r="E70" t="str">
-        <x:v>https://doi.org/10.1140/epjqt/s40507-023-00166-1</x:v>
-      </x:c>
-      <x:c r="F70" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="71">
-      <x:c r="A71" t="str">
-        <x:v>Offline Quantum Reinforcement Learning in a Conservative Manner</x:v>
-      </x:c>
-      <x:c r="B71" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C71" t="str">
-        <x:v>Proceedings of the AAAI Conference on Artificial Intelligence</x:v>
-      </x:c>
-      <x:c r="D71" t="str">
-        <x:v>Zhihao Cheng, Kaining Zhang, Li Shen, Dacheng Tao</x:v>
-      </x:c>
-      <x:c r="E71" t="str">
-        <x:v>https://doi.org/10.1609/aaai.v37i6.25872</x:v>
-      </x:c>
-      <x:c r="F71" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="72">
-      <x:c r="A72" t="str">
-        <x:v>Asynchronous training of quantum reinforcement learning</x:v>
-      </x:c>
-      <x:c r="B72" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C72" t="str">
-        <x:v>ScienceDirect</x:v>
-      </x:c>
-      <x:c r="D72" t="str">
-        <x:v>Samuel Yen-Chi Chen</x:v>
-      </x:c>
-      <x:c r="E72" t="str">
-        <x:v>https://doi.org/10.1016/j.procs.2023.08.171</x:v>
-      </x:c>
-      <x:c r="F72" t="str">
-        <x:v>QRL</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="73">
-      <x:c r="A73" t="str">
-        <x:v>Blockchain Based Optimized Energy Trading for E-Mobility Using Quantum Reinforcement Learning</x:v>
-      </x:c>
-      <x:c r="B73" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C73" t="str">
-        <x:v>IEEE</x:v>
-      </x:c>
-      <x:c r="D73" t="str">
-        <x:v>Manoj Kumar; Upasana Dohare; Sushil Kumar; Neeraj Kumar</x:v>
-      </x:c>
-      <x:c r="E73" t="str">
-        <x:v>https://doi.org/10.1109/TVT.2022.3225524</x:v>
       </x:c>
       <x:c r="F73" t="str">
         <x:v>QRL</x:v>
@@ -1796,19 +1796,19 @@
     </x:row>
     <x:row r="74">
       <x:c r="A74" t="str">
-        <x:v>Efficient Dimensionality Reduction Strategies for Quantum Reinforcement Learning</x:v>
+        <x:v>Reinforcement learning-based architecture search for quantum machine learning</x:v>
       </x:c>
       <x:c r="B74" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="C74" t="str">
-        <x:v>IEEE</x:v>
+        <x:v>arXiv</x:v>
       </x:c>
       <x:c r="D74" t="str">
-        <x:v>Eva Andrés; M. P. Cuéllar; G. Navarro</x:v>
+        <x:v>Rapp, Frederic, David A. Kreplin, and Marco Roth.</x:v>
       </x:c>
       <x:c r="E74" t="str">
-        <x:v>https://doi.org/10.1109/ACCESS.2023.3318173</x:v>
+        <x:v>https://arxiv.org/abs/2406.02717</x:v>
       </x:c>
       <x:c r="F74" t="str">
         <x:v>QRL</x:v>
@@ -1816,19 +1816,19 @@
     </x:row>
     <x:row r="75">
       <x:c r="A75" t="str">
-        <x:v>Deep reinforcement learning for quantum multiparameter estimation</x:v>
+        <x:v>Attention-Based Deep Reinforcement Learning for Qubit Allocation in Modular Quantum Architectures.</x:v>
       </x:c>
       <x:c r="B75" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="C75" t="str">
-        <x:v>SPIE</x:v>
+        <x:v>arXiv</x:v>
       </x:c>
       <x:c r="D75" t="str">
-        <x:v>Valeria Cimini, Mauro Valeri, Emanuele Polino, Simone Piacentini, Francesco Ceccarelli, Giacomo Corrielli, Nicolò Spagnolo, Roberto Osellame, Fabio Sciarrino</x:v>
+        <x:v>Russo, Enrico, et al.</x:v>
       </x:c>
       <x:c r="E75" t="str">
-        <x:v>https://doi.org/10.1117/1.AP.5.1.016005</x:v>
+        <x:v>https://arxiv.org/abs/2406.11452</x:v>
       </x:c>
       <x:c r="F75" t="str">
         <x:v>QRL</x:v>
@@ -1836,19 +1836,19 @@
     </x:row>
     <x:row r="76">
       <x:c r="A76" t="str">
-        <x:v>Approximate Autonomous Quantum Error Correction with Reinforcement Learning</x:v>
+        <x:v>Quantum reinforcement learning via policy iteration</x:v>
       </x:c>
       <x:c r="B76" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C76" t="str">
-        <x:v>Physical Review Letters</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D76" t="str">
-        <x:v>Yexiong Zeng, Zheng-Yang Zhou, Enrico Rinaldi, Clemens Gneiting, and Franco Nori</x:v>
+        <x:v>El Amine Cherrat, Iordanis Kerenidis, Anupam Prakash </x:v>
       </x:c>
       <x:c r="E76" t="str">
-        <x:v>https://doi.org/10.1103/PhysRevLett.131.050601</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00116-1</x:v>
       </x:c>
       <x:c r="F76" t="str">
         <x:v>QRL</x:v>
@@ -1856,7 +1856,7 @@
     </x:row>
     <x:row r="77">
       <x:c r="A77" t="str">
-        <x:v>Quantum reinforcement learning</x:v>
+        <x:v>Policy gradients using variational quantum circuits</x:v>
       </x:c>
       <x:c r="B77" t="n">
         <x:v>2023</x:v>
@@ -1865,10 +1865,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D77" t="str">
-        <x:v>Niels M. P. Neumann, Paolo B. U. L. de Heer &amp; Frank Phillipson </x:v>
+        <x:v>André Sequeira, Luis Paulo Santos, Luis Soares Barbosa </x:v>
       </x:c>
       <x:c r="E77" t="str">
-        <x:v>https://doi.org/10.1007/s11128-023-03867-9</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00101-8</x:v>
       </x:c>
       <x:c r="F77" t="str">
         <x:v>QRL</x:v>
@@ -1876,19 +1876,19 @@
     </x:row>
     <x:row r="78">
       <x:c r="A78" t="str">
-        <x:v>Quantum Reinforcement Learning for Quantum Architecture Search</x:v>
+        <x:v>Robustness of quantum reinforcement learning under hardware errors</x:v>
       </x:c>
       <x:c r="B78" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C78" t="str">
-        <x:v>ACM</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D78" t="str">
-        <x:v>Samuel Yen-Chi Chen</x:v>
+        <x:v>Andrea Skolik, Stefano Mangini, Thomas Bäck, Chiara Macchiavello &amp; Vedran Dunjko </x:v>
       </x:c>
       <x:c r="E78" t="str">
-        <x:v>https://doi.org/10.1145/3588983.3596692</x:v>
+        <x:v>https://doi.org/10.1140/epjqt/s40507-023-00166-1</x:v>
       </x:c>
       <x:c r="F78" t="str">
         <x:v>QRL</x:v>
@@ -1896,19 +1896,19 @@
     </x:row>
     <x:row r="79">
       <x:c r="A79" t="str">
-        <x:v>Quantum Deep Recurrent Reinforcement Learning</x:v>
+        <x:v>Offline Quantum Reinforcement Learning in a Conservative Manner</x:v>
       </x:c>
       <x:c r="B79" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C79" t="str">
-        <x:v>IEEE</x:v>
+        <x:v>Proceedings of the AAAI Conference on Artificial Intelligence</x:v>
       </x:c>
       <x:c r="D79" t="str">
-        <x:v>Samuel Yen-Chi Chen</x:v>
+        <x:v>Zhihao Cheng, Kaining Zhang, Li Shen, Dacheng Tao</x:v>
       </x:c>
       <x:c r="E79" t="str">
-        <x:v>https://doi.org/10.1109/ICASSP49357.2023.10096981</x:v>
+        <x:v>https://doi.org/10.1609/aaai.v37i6.25872</x:v>
       </x:c>
       <x:c r="F79" t="str">
         <x:v>QRL</x:v>
@@ -1916,19 +1916,19 @@
     </x:row>
     <x:row r="80">
       <x:c r="A80" t="str">
-        <x:v>Differentiable Quantum Architecture Search for Quantum Reinforcement Learning</x:v>
+        <x:v>Asynchronous training of quantum reinforcement learning</x:v>
       </x:c>
       <x:c r="B80" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C80" t="str">
-        <x:v>IEEE</x:v>
+        <x:v>ScienceDirect</x:v>
       </x:c>
       <x:c r="D80" t="str">
-        <x:v>Yize Sun; Yunpu Ma; Volker Tresp</x:v>
+        <x:v>Samuel Yen-Chi Chen</x:v>
       </x:c>
       <x:c r="E80" t="str">
-        <x:v>https://doi.org/10.1109/QCE57702.2023.10177</x:v>
+        <x:v>https://doi.org/10.1016/j.procs.2023.08.171</x:v>
       </x:c>
       <x:c r="F80" t="str">
         <x:v>QRL</x:v>
@@ -1936,7 +1936,7 @@
     </x:row>
     <x:row r="81">
       <x:c r="A81" t="str">
-        <x:v>Quantum Multi-Agent Reinforcement Learning for Autonomous Mobility Cooperation</x:v>
+        <x:v>Blockchain Based Optimized Energy Trading for E-Mobility Using Quantum Reinforcement Learning</x:v>
       </x:c>
       <x:c r="B81" t="n">
         <x:v>2023</x:v>
@@ -1945,10 +1945,10 @@
         <x:v>IEEE</x:v>
       </x:c>
       <x:c r="D81" t="str">
-        <x:v>Soohyun Park; Jae Pyoung Kim; Chanyoung Park; Soyi Jung; Joongheon Kim</x:v>
+        <x:v>Manoj Kumar; Upasana Dohare; Sushil Kumar; Neeraj Kumar</x:v>
       </x:c>
       <x:c r="E81" t="str">
-        <x:v>https://doi.org/10.1109/MCOM.020.2300199</x:v>
+        <x:v>https://doi.org/10.1109/TVT.2022.3225524</x:v>
       </x:c>
       <x:c r="F81" t="str">
         <x:v>QRL</x:v>
@@ -1956,19 +1956,19 @@
     </x:row>
     <x:row r="82">
       <x:c r="A82" t="str">
-        <x:v>Quantum reinforcement learning in the presence of thermal dissipation</x:v>
+        <x:v>Efficient Dimensionality Reduction Strategies for Quantum Reinforcement Learning</x:v>
       </x:c>
       <x:c r="B82" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C82" t="str">
-        <x:v>APS</x:v>
+        <x:v>IEEE</x:v>
       </x:c>
       <x:c r="D82" t="str">
-        <x:v>María Laura Olivera-Atencio, Lucas Lamata, Manuel Morillo, and Jesús Casado-Pascual</x:v>
+        <x:v>Eva Andrés; M. P. Cuéllar; G. Navarro</x:v>
       </x:c>
       <x:c r="E82" t="str">
-        <x:v>https://doi.org/10.1103/PhysRevE.108.014128</x:v>
+        <x:v>https://doi.org/10.1109/ACCESS.2023.3318173</x:v>
       </x:c>
       <x:c r="F82" t="str">
         <x:v>QRL</x:v>
@@ -1976,19 +1976,19 @@
     </x:row>
     <x:row r="83">
       <x:c r="A83" t="str">
-        <x:v>Quantum Multi-Agent Meta Reinforcement Learning</x:v>
+        <x:v>Deep reinforcement learning for quantum multiparameter estimation</x:v>
       </x:c>
       <x:c r="B83" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C83" t="str">
-        <x:v>Proceedings of the AAAI Conference on Artificial Intelligence</x:v>
+        <x:v>SPIE</x:v>
       </x:c>
       <x:c r="D83" t="str">
-        <x:v>Won Joon Yun, Jihong Park, Joongheon Kim</x:v>
+        <x:v>Valeria Cimini, Mauro Valeri, Emanuele Polino, Simone Piacentini, Francesco Ceccarelli, Giacomo Corrielli, Nicolò Spagnolo, Roberto Osellame, Fabio Sciarrino</x:v>
       </x:c>
       <x:c r="E83" t="str">
-        <x:v>https://doi.org/10.1609/aaai.v37i9.26313</x:v>
+        <x:v>https://doi.org/10.1117/1.AP.5.1.016005</x:v>
       </x:c>
       <x:c r="F83" t="str">
         <x:v>QRL</x:v>
@@ -1996,19 +1996,19 @@
     </x:row>
     <x:row r="84">
       <x:c r="A84" t="str">
-        <x:v>Realizing a deep reinforcement learning agent for real-time quantum feedback</x:v>
+        <x:v>Approximate Autonomous Quantum Error Correction with Reinforcement Learning</x:v>
       </x:c>
       <x:c r="B84" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C84" t="str">
-        <x:v>Nature Communications</x:v>
+        <x:v>Physical Review Letters</x:v>
       </x:c>
       <x:c r="D84" t="str">
-        <x:v>Kevin Reuer, Jonas Landgraf, Thomas Fösel, James O’Sullivan, Liberto Beltrán, Abdulkadir Akin, Graham J. Norris, Ants Remm, Michael Kerschbaum, Jean-Claude Besse, Florian Marquardt, Andreas Wallraff &amp; Christopher Eichler</x:v>
+        <x:v>Yexiong Zeng, Zheng-Yang Zhou, Enrico Rinaldi, Clemens Gneiting, and Franco Nori</x:v>
       </x:c>
       <x:c r="E84" t="str">
-        <x:v>https://doi.org/10.1038/s41467-023-42901-3</x:v>
+        <x:v>https://doi.org/10.1103/PhysRevLett.131.050601</x:v>
       </x:c>
       <x:c r="F84" t="str">
         <x:v>QRL</x:v>
@@ -2016,19 +2016,19 @@
     </x:row>
     <x:row r="85">
       <x:c r="A85" t="str">
-        <x:v>Quafu-RL: The Cloud Quantum Computers based Quantum Reinforcement Learning</x:v>
+        <x:v>Quantum reinforcement learning</x:v>
       </x:c>
       <x:c r="B85" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C85" t="str">
-        <x:v>arXiv</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D85" t="str">
-        <x:v>BAQIS Quafu Group</x:v>
+        <x:v>Niels M. P. Neumann, Paolo B. U. L. de Heer &amp; Frank Phillipson </x:v>
       </x:c>
       <x:c r="E85" t="str">
-        <x:v>https://doi.org/10.48550/arXiv.2305.17966</x:v>
+        <x:v>https://doi.org/10.1007/s11128-023-03867-9</x:v>
       </x:c>
       <x:c r="F85" t="str">
         <x:v>QRL</x:v>
@@ -2036,19 +2036,19 @@
     </x:row>
     <x:row r="86">
       <x:c r="A86" t="str">
-        <x:v>Provably Efficient Exploration in Quantum Reinforcement Learning with Logarithmic Worst-Case Regret</x:v>
+        <x:v>Quantum Reinforcement Learning for Quantum Architecture Search</x:v>
       </x:c>
       <x:c r="B86" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C86" t="str">
-        <x:v>arXiv</x:v>
+        <x:v>ACM</x:v>
       </x:c>
       <x:c r="D86" t="str">
-        <x:v>Han Zhong, Jiachen Hu, Yecheng Xue, Tongyang Li, Liwei Wang</x:v>
+        <x:v>Samuel Yen-Chi Chen</x:v>
       </x:c>
       <x:c r="E86" t="str">
-        <x:v>https://doi.org/10.48550/arXiv.2302.10796</x:v>
+        <x:v>https://doi.org/10.1145/3588983.3596692</x:v>
       </x:c>
       <x:c r="F86" t="str">
         <x:v>QRL</x:v>
@@ -2056,19 +2056,19 @@
     </x:row>
     <x:row r="87">
       <x:c r="A87" t="str">
-        <x:v>Safe reinforcement learning under temporal logic with reward design and quantum action selection</x:v>
+        <x:v>Quantum Deep Recurrent Reinforcement Learning</x:v>
       </x:c>
       <x:c r="B87" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C87" t="str">
-        <x:v>Scientific Reports</x:v>
+        <x:v>IEEE</x:v>
       </x:c>
       <x:c r="D87" t="str">
-        <x:v>Mingyu Cai, Shaoping Xiao, Junchao Li &amp; Zhen Kan</x:v>
+        <x:v>Samuel Yen-Chi Chen</x:v>
       </x:c>
       <x:c r="E87" t="str">
-        <x:v>https://doi.org/10.1038/s41598-023-28582-4</x:v>
+        <x:v>https://doi.org/10.1109/ICASSP49357.2023.10096981</x:v>
       </x:c>
       <x:c r="F87" t="str">
         <x:v>QRL</x:v>
@@ -2076,19 +2076,19 @@
     </x:row>
     <x:row r="88">
       <x:c r="A88" t="str">
-        <x:v>Self-correcting quantum many-body control using reinforcement learning with tensor networks</x:v>
+        <x:v>Differentiable Quantum Architecture Search for Quantum Reinforcement Learning</x:v>
       </x:c>
       <x:c r="B88" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C88" t="str">
-        <x:v>Nature Machine Intelligence</x:v>
+        <x:v>IEEE</x:v>
       </x:c>
       <x:c r="D88" t="str">
-        <x:v>Friederike Metz &amp; Marin Bukov</x:v>
+        <x:v>Yize Sun; Yunpu Ma; Volker Tresp</x:v>
       </x:c>
       <x:c r="E88" t="str">
-        <x:v>https://doi.org/10.1038/s42256-023-00687-5</x:v>
+        <x:v>https://doi.org/10.1109/QCE57702.2023.10177</x:v>
       </x:c>
       <x:c r="F88" t="str">
         <x:v>QRL</x:v>
@@ -2096,19 +2096,19 @@
     </x:row>
     <x:row r="89">
       <x:c r="A89" t="str">
-        <x:v>Model-free optimization of power/efficiency tradeoffs in quantum thermal machines using reinforcement learning</x:v>
+        <x:v>Quantum Multi-Agent Reinforcement Learning for Autonomous Mobility Cooperation</x:v>
       </x:c>
       <x:c r="B89" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C89" t="str">
-        <x:v>Paolo A Erdman, Frank Noé</x:v>
+        <x:v>IEEE</x:v>
       </x:c>
       <x:c r="D89" t="str">
-        <x:v>PNAS Nexus</x:v>
+        <x:v>Soohyun Park; Jae Pyoung Kim; Chanyoung Park; Soyi Jung; Joongheon Kim</x:v>
       </x:c>
       <x:c r="E89" t="str">
-        <x:v>https://doi.org/10.1093/pnasnexus/pgad248</x:v>
+        <x:v>https://doi.org/10.1109/MCOM.020.2300199</x:v>
       </x:c>
       <x:c r="F89" t="str">
         <x:v>QRL</x:v>
@@ -2116,19 +2116,19 @@
     </x:row>
     <x:row r="90">
       <x:c r="A90" t="str">
-        <x:v>A Survey on Quantum Reinforcement Learning</x:v>
+        <x:v>Quantum reinforcement learning in the presence of thermal dissipation</x:v>
       </x:c>
       <x:c r="B90" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C90" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>APS</x:v>
       </x:c>
       <x:c r="D90" t="str">
-        <x:v>Nico Meyer, Christian Ufrecht, Maniraman Periyasamy, Daniel D. Scherer, Axel Plinge, Christopher Mutschler</x:v>
+        <x:v>María Laura Olivera-Atencio, Lucas Lamata, Manuel Morillo, and Jesús Casado-Pascual</x:v>
       </x:c>
       <x:c r="E90" t="str">
-        <x:v>https://arxiv.org/abs/2211.03464</x:v>
+        <x:v>https://doi.org/10.1103/PhysRevE.108.014128</x:v>
       </x:c>
       <x:c r="F90" t="str">
         <x:v>QRL</x:v>
@@ -2136,19 +2136,19 @@
     </x:row>
     <x:row r="91">
       <x:c r="A91" t="str">
-        <x:v>Quantum reinforcement learning: the maze problem</x:v>
+        <x:v>Quantum Multi-Agent Meta Reinforcement Learning</x:v>
       </x:c>
       <x:c r="B91" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C91" t="str">
-        <x:v>Quantum Machine Intelligence</x:v>
+        <x:v>Proceedings of the AAAI Conference on Artificial Intelligence</x:v>
       </x:c>
       <x:c r="D91" t="str">
-        <x:v>Nicola Dalla Pozza, Lorenzo Buffoni, …Filippo Caruso</x:v>
+        <x:v>Won Joon Yun, Jihong Park, Joongheon Kim</x:v>
       </x:c>
       <x:c r="E91" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s42484-022-00068-y</x:v>
+        <x:v>https://doi.org/10.1609/aaai.v37i9.26313</x:v>
       </x:c>
       <x:c r="F91" t="str">
         <x:v>QRL</x:v>
@@ -2156,19 +2156,19 @@
     </x:row>
     <x:row r="92">
       <x:c r="A92" t="str">
-        <x:v>Variational quantum reinforcement learning via evolutionary optimization</x:v>
+        <x:v>Realizing a deep reinforcement learning agent for real-time quantum feedback</x:v>
       </x:c>
       <x:c r="B92" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C92" t="str">
-        <x:v>IOP Publishing Ltd </x:v>
+        <x:v>Nature Communications</x:v>
       </x:c>
       <x:c r="D92" t="str">
-        <x:v>Samuel Yen-Chi Chen, Chih-Min Huang2, Chia-Wei Hsing, Hsi-Sheng Goan and Ying-Jer Kao</x:v>
+        <x:v>Kevin Reuer, Jonas Landgraf, Thomas Fösel, James O’Sullivan, Liberto Beltrán, Abdulkadir Akin, Graham J. Norris, Ants Remm, Michael Kerschbaum, Jean-Claude Besse, Florian Marquardt, Andreas Wallraff &amp; Christopher Eichler</x:v>
       </x:c>
       <x:c r="E92" t="str">
-        <x:v>https://iopscience.iop.org/article/10.1088/2632-2153/ac4559/meta</x:v>
+        <x:v>https://doi.org/10.1038/s41467-023-42901-3</x:v>
       </x:c>
       <x:c r="F92" t="str">
         <x:v>QRL</x:v>
@@ -2176,19 +2176,19 @@
     </x:row>
     <x:row r="93">
       <x:c r="A93" t="str">
-        <x:v>On the Use of Quantum Reinforcement Learning in Energy-Efficiency Scenarios</x:v>
+        <x:v>Quafu-RL: The Cloud Quantum Computers based Quantum Reinforcement Learning</x:v>
       </x:c>
       <x:c r="B93" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C93" t="str">
-        <x:v>Energy Efficiency and Energy Consumption Modelling Using Artificial Neural Networks</x:v>
+        <x:v>arXiv</x:v>
       </x:c>
       <x:c r="D93" t="str">
-        <x:v>Eva Andrés, Manuel Pegalajar Cuéllar and Gabriel Navarro</x:v>
+        <x:v>BAQIS Quafu Group</x:v>
       </x:c>
       <x:c r="E93" t="str">
-        <x:v>https://www.mdpi.com/1996-1073/15/16/6034</x:v>
+        <x:v>https://doi.org/10.48550/arXiv.2305.17966</x:v>
       </x:c>
       <x:c r="F93" t="str">
         <x:v>QRL</x:v>
@@ -2196,19 +2196,19 @@
     </x:row>
     <x:row r="94">
       <x:c r="A94" t="str">
-        <x:v>Unentangled quantum reinforcement learning agents in the OpenAI Gym</x:v>
+        <x:v>Provably Efficient Exploration in Quantum Reinforcement Learning with Logarithmic Worst-Case Regret</x:v>
       </x:c>
       <x:c r="B94" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C94" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>arXiv</x:v>
       </x:c>
       <x:c r="D94" t="str">
-        <x:v>Jen-Yueh Hsiao, Yuxuan Du, Wei-Yin Chiang, Min-Hsiu Hsieh, Hsi-Sheng Goan</x:v>
+        <x:v>Han Zhong, Jiachen Hu, Yecheng Xue, Tongyang Li, Liwei Wang</x:v>
       </x:c>
       <x:c r="E94" t="str">
-        <x:v>https://arxiv.org/abs/2203.14348</x:v>
+        <x:v>https://doi.org/10.48550/arXiv.2302.10796</x:v>
       </x:c>
       <x:c r="F94" t="str">
         <x:v>QRL</x:v>
@@ -2216,19 +2216,19 @@
     </x:row>
     <x:row r="95">
       <x:c r="A95" t="str">
-        <x:v>Model-Free Quantum Control with Reinforcement Learning</x:v>
+        <x:v>Safe reinforcement learning under temporal logic with reward design and quantum action selection</x:v>
       </x:c>
       <x:c r="B95" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C95" t="str">
-        <x:v>Phys. Rev. X 12</x:v>
+        <x:v>Scientific Reports</x:v>
       </x:c>
       <x:c r="D95" t="str">
-        <x:v>V. V. Sivak, A. Eickbusch, H. Liu, B. Royer, I. Tsioutsios, and M. H. Devoret</x:v>
+        <x:v>Mingyu Cai, Shaoping Xiao, Junchao Li &amp; Zhen Kan</x:v>
       </x:c>
       <x:c r="E95" t="str">
-        <x:v>https://journals.aps.org/prx/abstract/10.1103/PhysRevX.12.011059</x:v>
+        <x:v>https://doi.org/10.1038/s41598-023-28582-4</x:v>
       </x:c>
       <x:c r="F95" t="str">
         <x:v>QRL</x:v>
@@ -2236,19 +2236,19 @@
     </x:row>
     <x:row r="96">
       <x:c r="A96" t="str">
-        <x:v>An Approach Based on Quantum Reinforcement Learning for Navigation Problems</x:v>
+        <x:v>Self-correcting quantum many-body control using reinforcement learning with tensor networks</x:v>
       </x:c>
       <x:c r="B96" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C96" t="str">
-        <x:v>2022 International Conference on Data Analytics for Business and Industry (ICDABI)</x:v>
+        <x:v>Nature Machine Intelligence</x:v>
       </x:c>
       <x:c r="D96" t="str">
-        <x:v>Niyazi Furkan Bar; Hasan Yetis; Mehmet Karakose</x:v>
+        <x:v>Friederike Metz &amp; Marin Bukov</x:v>
       </x:c>
       <x:c r="E96" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/10041570</x:v>
+        <x:v>https://doi.org/10.1038/s42256-023-00687-5</x:v>
       </x:c>
       <x:c r="F96" t="str">
         <x:v>QRL</x:v>
@@ -2256,19 +2256,19 @@
     </x:row>
     <x:row r="97">
       <x:c r="A97" t="str">
-        <x:v>Curriculum-Based Deep Reinforcement Learning for Quantum Control</x:v>
+        <x:v>Model-free optimization of power/efficiency tradeoffs in quantum thermal machines using reinforcement learning</x:v>
       </x:c>
       <x:c r="B97" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C97" t="str">
-        <x:v>IEEE Transactions on Neural Networks and Learning Systems</x:v>
+        <x:v>Paolo A Erdman, Frank Noé</x:v>
       </x:c>
       <x:c r="D97" t="str">
-        <x:v>Hailan Ma; Daoyi Dong; Steven X. Ding; Chunlin Chen</x:v>
+        <x:v>PNAS Nexus</x:v>
       </x:c>
       <x:c r="E97" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9732235</x:v>
+        <x:v>https://doi.org/10.1093/pnasnexus/pgad248</x:v>
       </x:c>
       <x:c r="F97" t="str">
         <x:v>QRL</x:v>
@@ -2276,19 +2276,19 @@
     </x:row>
     <x:row r="98">
       <x:c r="A98" t="str">
-        <x:v>A quantum system control method based on enhanced reinforcement learning</x:v>
+        <x:v>A Survey on Quantum Reinforcement Learning</x:v>
       </x:c>
       <x:c r="B98" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C98" t="str">
-        <x:v>Data analytics and machine learning</x:v>
+        <x:v>arxiv</x:v>
       </x:c>
       <x:c r="D98" t="str">
-        <x:v>Wenjie Liu, Bosi Wang, …Mohammed Zidan</x:v>
+        <x:v>Nico Meyer, Christian Ufrecht, Maniraman Periyasamy, Daniel D. Scherer, Axel Plinge, Christopher Mutschler</x:v>
       </x:c>
       <x:c r="E98" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s00500-022-07179-5</x:v>
+        <x:v>https://arxiv.org/abs/2211.03464</x:v>
       </x:c>
       <x:c r="F98" t="str">
         <x:v>QRL</x:v>
@@ -2296,19 +2296,19 @@
     </x:row>
     <x:row r="99">
       <x:c r="A99" t="str">
-        <x:v>Deep Reinforcement Learning for Quantum Hamiltonian Engineering</x:v>
+        <x:v>Quantum reinforcement learning: the maze problem</x:v>
       </x:c>
       <x:c r="B99" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C99" t="str">
-        <x:v>Phys. Rev. Applied 18</x:v>
+        <x:v>Quantum Machine Intelligence</x:v>
       </x:c>
       <x:c r="D99" t="str">
-        <x:v>Pai Peng (彭湃), Xiaoyang Huang, Chao Yin, Linta Joseph, Chandrasekhar Ramanathan, and Paola Cappellaro</x:v>
+        <x:v>Nicola Dalla Pozza, Lorenzo Buffoni, …Filippo Caruso</x:v>
       </x:c>
       <x:c r="E99" t="str">
-        <x:v>https://journals.aps.org/prapplied/abstract/10.1103/PhysRevApplied.18.024033</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s42484-022-00068-y</x:v>
       </x:c>
       <x:c r="F99" t="str">
         <x:v>QRL</x:v>
@@ -2316,19 +2316,19 @@
     </x:row>
     <x:row r="100">
       <x:c r="A100" t="str">
-        <x:v>Parameter estimation in quantum sensing based on deep reinforcement learning</x:v>
+        <x:v>Variational quantum reinforcement learning via evolutionary optimization</x:v>
       </x:c>
       <x:c r="B100" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C100" t="str">
-        <x:v>npj Quantum Information</x:v>
+        <x:v>IOP Publishing Ltd </x:v>
       </x:c>
       <x:c r="D100" t="str">
-        <x:v>      Tailong Xiao, Jianping Fan &amp; Guihua Zeng   </x:v>
+        <x:v>Samuel Yen-Chi Chen, Chih-Min Huang2, Chia-Wei Hsing, Hsi-Sheng Goan and Ying-Jer Kao</x:v>
       </x:c>
       <x:c r="E100" t="str">
-        <x:v>https://www.nature.com/articles/s41534-021-00513-z</x:v>
+        <x:v>https://iopscience.iop.org/article/10.1088/2632-2153/ac4559/meta</x:v>
       </x:c>
       <x:c r="F100" t="str">
         <x:v>QRL</x:v>
@@ -2336,19 +2336,19 @@
     </x:row>
     <x:row r="101">
       <x:c r="A101" t="str">
-        <x:v>Quantum Deep Reinforcement Learning for Robot Navigation Tasks</x:v>
+        <x:v>On the Use of Quantum Reinforcement Learning in Energy-Efficiency Scenarios</x:v>
       </x:c>
       <x:c r="B101" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C101" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>Energy Efficiency and Energy Consumption Modelling Using Artificial Neural Networks</x:v>
       </x:c>
       <x:c r="D101" t="str">
-        <x:v>Hans Hohenfeld, Dirk Heimann, Felix Wiebe, Frank Kirchner</x:v>
+        <x:v>Eva Andrés, Manuel Pegalajar Cuéllar and Gabriel Navarro</x:v>
       </x:c>
       <x:c r="E101" t="str">
-        <x:v>https://arxiv.org/abs/2202.12180</x:v>
+        <x:v>https://www.mdpi.com/1996-1073/15/16/6034</x:v>
       </x:c>
       <x:c r="F101" t="str">
         <x:v>QRL</x:v>
@@ -2356,19 +2356,19 @@
     </x:row>
     <x:row r="102">
       <x:c r="A102" t="str">
-        <x:v>Robust optimization for quantum reinforcement learning control using partial observations</x:v>
+        <x:v>Unentangled quantum reinforcement learning agents in the OpenAI Gym</x:v>
       </x:c>
       <x:c r="B102" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C102" t="str">
-        <x:v>Phys. Rev. A 105</x:v>
+        <x:v>arxiv</x:v>
       </x:c>
       <x:c r="D102" t="str">
-        <x:v>Chen Jiang, Yu Pan, Zheng-Guang Wu, Qing Gao, and Daoyi Dong</x:v>
+        <x:v>Jen-Yueh Hsiao, Yuxuan Du, Wei-Yin Chiang, Min-Hsiu Hsieh, Hsi-Sheng Goan</x:v>
       </x:c>
       <x:c r="E102" t="str">
-        <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.105.062443</x:v>
+        <x:v>https://arxiv.org/abs/2203.14348</x:v>
       </x:c>
       <x:c r="F102" t="str">
         <x:v>QRL</x:v>
@@ -2376,19 +2376,19 @@
     </x:row>
     <x:row r="103">
       <x:c r="A103" t="str">
-        <x:v>Using Reinforcement Learning to Perform Qubit Routing in Quantum Compilers</x:v>
+        <x:v>Model-Free Quantum Control with Reinforcement Learning</x:v>
       </x:c>
       <x:c r="B103" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C103" t="str">
-        <x:v>ACM Transactions on Quantum Computing</x:v>
+        <x:v>Phys. Rev. X 12</x:v>
       </x:c>
       <x:c r="D103" t="str">
-        <x:v>Matteo G. Pozzi, Steven J. Herbert, Akash Sengupta, Robert D. Mullins</x:v>
+        <x:v>V. V. Sivak, A. Eickbusch, H. Liu, B. Royer, I. Tsioutsios, and M. H. Devoret</x:v>
       </x:c>
       <x:c r="E103" t="str">
-        <x:v>https://dl.acm.org/doi/full/10.1145/3520434</x:v>
+        <x:v>https://journals.aps.org/prx/abstract/10.1103/PhysRevX.12.011059</x:v>
       </x:c>
       <x:c r="F103" t="str">
         <x:v>QRL</x:v>
@@ -2396,19 +2396,19 @@
     </x:row>
     <x:row r="104">
       <x:c r="A104" t="str">
-        <x:v>Quantum reinforcement learning method and application based on value function</x:v>
+        <x:v>An Approach Based on Quantum Reinforcement Learning for Navigation Problems</x:v>
       </x:c>
       <x:c r="B104" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C104" t="str">
-        <x:v>IFAC-PapersOnLine</x:v>
+        <x:v>2022 International Conference on Data Analytics for Business and Industry (ICDABI)</x:v>
       </x:c>
       <x:c r="D104" t="str">
-        <x:v>Yi-Pei Liu *, Qing-Shan Jia *, Xu Wang </x:v>
+        <x:v>Niyazi Furkan Bar; Hasan Yetis; Mehmet Karakose</x:v>
       </x:c>
       <x:c r="E104" t="str">
-        <x:v>https://www.sciencedirect.com/science/article/pii/S2405896322011508#aep-article-footnote-id1</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/10041570</x:v>
       </x:c>
       <x:c r="F104" t="str">
         <x:v>QRL</x:v>
@@ -2416,19 +2416,19 @@
     </x:row>
     <x:row r="105">
       <x:c r="A105" t="str">
-        <x:v>Identifying optimal cycles in quantum thermal machines with reinforcement-learning</x:v>
+        <x:v>Curriculum-Based Deep Reinforcement Learning for Quantum Control</x:v>
       </x:c>
       <x:c r="B105" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C105" t="str">
-        <x:v>npj Quantum Information</x:v>
+        <x:v>IEEE Transactions on Neural Networks and Learning Systems</x:v>
       </x:c>
       <x:c r="D105" t="str">
-        <x:v>Paolo A. Erdman &amp; Frank Noé </x:v>
+        <x:v>Hailan Ma; Daoyi Dong; Steven X. Ding; Chunlin Chen</x:v>
       </x:c>
       <x:c r="E105" t="str">
-        <x:v>https://www.nature.com/articles/s41534-021-00512-0</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9732235</x:v>
       </x:c>
       <x:c r="F105" t="str">
         <x:v>QRL</x:v>
@@ -2436,19 +2436,19 @@
     </x:row>
     <x:row r="106">
       <x:c r="A106" t="str">
-        <x:v>Quantum Policy Iteration via Amplitude Estimation and Grover Search -- Towards Quantum Advantage for Reinforcement Learning</x:v>
+        <x:v>A quantum system control method based on enhanced reinforcement learning</x:v>
       </x:c>
       <x:c r="B106" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C106" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>Data analytics and machine learning</x:v>
       </x:c>
       <x:c r="D106" t="str">
-        <x:v>Simon Wiedemann, Daniel Hein, Steffen Udluft, Christian Mendl</x:v>
+        <x:v>Wenjie Liu, Bosi Wang, …Mohammed Zidan</x:v>
       </x:c>
       <x:c r="E106" t="str">
-        <x:v>https://arxiv.org/abs/2206.04741</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s00500-022-07179-5</x:v>
       </x:c>
       <x:c r="F106" t="str">
         <x:v>QRL</x:v>
@@ -2456,19 +2456,19 @@
     </x:row>
     <x:row r="107">
       <x:c r="A107" t="str">
-        <x:v>Quantum Reinforcement Learning for Solving a Stochastic Frozen Lake Environment and the Impact of Quantum Architecture Choices</x:v>
+        <x:v>Deep Reinforcement Learning for Quantum Hamiltonian Engineering</x:v>
       </x:c>
       <x:c r="B107" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C107" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>Phys. Rev. Applied 18</x:v>
       </x:c>
       <x:c r="D107" t="str">
-        <x:v>Theodora-Augustina Drăgan, Maureen Monnet, Christian B. Mendl, Jeanette Miriam Lorenz</x:v>
+        <x:v>Pai Peng (彭湃), Xiaoyang Huang, Chao Yin, Linta Joseph, Chandrasekhar Ramanathan, and Paola Cappellaro</x:v>
       </x:c>
       <x:c r="E107" t="str">
-        <x:v>https://arxiv.org/abs/2212.07932</x:v>
+        <x:v>https://journals.aps.org/prapplied/abstract/10.1103/PhysRevApplied.18.024033</x:v>
       </x:c>
       <x:c r="F107" t="str">
         <x:v>QRL</x:v>
@@ -2476,19 +2476,19 @@
     </x:row>
     <x:row r="108">
       <x:c r="A108" t="str">
-        <x:v>Quantum Multi-Agent Reinforcement Learning via Variational Quantum Circuit Design</x:v>
+        <x:v>Parameter estimation in quantum sensing based on deep reinforcement learning</x:v>
       </x:c>
       <x:c r="B108" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C108" t="str">
-        <x:v>2022 IEEE 42nd International Conference on Distributed Computing Systems (ICDCS)</x:v>
+        <x:v>npj Quantum Information</x:v>
       </x:c>
       <x:c r="D108" t="str">
-        <x:v>Won Joon Yun; Yunseok Kwak; Jae Pyoung Kim; Hyunhee Cho; Soyi Jung; Jihong Park</x:v>
+        <x:v>      Tailong Xiao, Jianping Fan &amp; Guihua Zeng   </x:v>
       </x:c>
       <x:c r="E108" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9912289</x:v>
+        <x:v>https://www.nature.com/articles/s41534-021-00513-z</x:v>
       </x:c>
       <x:c r="F108" t="str">
         <x:v>QRL</x:v>
@@ -2496,19 +2496,19 @@
     </x:row>
     <x:row r="109">
       <x:c r="A109" t="str">
-        <x:v>Efficient and robust entanglement generation with deep reinforcement learning for quantum metrology</x:v>
+        <x:v>Quantum Deep Reinforcement Learning for Robot Navigation Tasks</x:v>
       </x:c>
       <x:c r="B109" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C109" t="str">
-        <x:v>New Journal of Physics (NJP)</x:v>
+        <x:v>arxiv</x:v>
       </x:c>
       <x:c r="D109" t="str">
-        <x:v>Yuxiang Qiu, Min Zhuang, Jiahao Huang and Chaohong Lee</x:v>
+        <x:v>Hans Hohenfeld, Dirk Heimann, Felix Wiebe, Frank Kirchner</x:v>
       </x:c>
       <x:c r="E109" t="str">
-        <x:v>https://iopscience.iop.org/article/10.1088/1367-2630/ac8285/meta</x:v>
+        <x:v>https://arxiv.org/abs/2202.12180</x:v>
       </x:c>
       <x:c r="F109" t="str">
         <x:v>QRL</x:v>
@@ -2516,19 +2516,19 @@
     </x:row>
     <x:row r="110">
       <x:c r="A110" t="str">
-        <x:v>NFT-Based Intelligence Networking for Connected and Autonomous Vehicles: A Quantum Reinforcement Learning Approach</x:v>
+        <x:v>Robust optimization for quantum reinforcement learning control using partial observations</x:v>
       </x:c>
       <x:c r="B110" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C110" t="str">
-        <x:v>IEEE Network</x:v>
+        <x:v>Phys. Rev. A 105</x:v>
       </x:c>
       <x:c r="D110" t="str">
-        <x:v>Yuzheng Ren; Renchao Xie; F. Richard Yu; Tao Huang; Yunjie Liu</x:v>
+        <x:v>Chen Jiang, Yu Pan, Zheng-Guang Wu, Qing Gao, and Daoyi Dong</x:v>
       </x:c>
       <x:c r="E110" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9852376</x:v>
+        <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.105.062443</x:v>
       </x:c>
       <x:c r="F110" t="str">
         <x:v>QRL</x:v>
@@ -2536,19 +2536,19 @@
     </x:row>
     <x:row r="111">
       <x:c r="A111" t="str">
-        <x:v>Quantum imaginary time evolution steered by reinforcement learning</x:v>
+        <x:v>Using Reinforcement Learning to Perform Qubit Routing in Quantum Compilers</x:v>
       </x:c>
       <x:c r="B111" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C111" t="str">
-        <x:v>Communications Physics volume</x:v>
+        <x:v>ACM Transactions on Quantum Computing</x:v>
       </x:c>
       <x:c r="D111" t="str">
-        <x:v>      Chenfeng Cao, Zheng An, Shi-Yao Hou, D. L. Zhou &amp; Bei Zeng   </x:v>
+        <x:v>Matteo G. Pozzi, Steven J. Herbert, Akash Sengupta, Robert D. Mullins</x:v>
       </x:c>
       <x:c r="E111" t="str">
-        <x:v>https://www.nature.com/articles/s42005-022-00837-y</x:v>
+        <x:v>https://dl.acm.org/doi/full/10.1145/3520434</x:v>
       </x:c>
       <x:c r="F111" t="str">
         <x:v>QRL</x:v>
@@ -2556,19 +2556,19 @@
     </x:row>
     <x:row r="112">
       <x:c r="A112" t="str">
-        <x:v>A tutorial on optimal control and reinforcement learning methods for quantum technologies</x:v>
+        <x:v>Quantum reinforcement learning method and application based on value function</x:v>
       </x:c>
       <x:c r="B112" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C112" t="str">
-        <x:v>Physics Letters A</x:v>
+        <x:v>IFAC-PapersOnLine</x:v>
       </x:c>
       <x:c r="D112" t="str">
-        <x:v>Luigi Giannelli a b, Sofia Sgroi d, Jonathon Brown d, Gheorghe Sorin Paraoanu e, Mauro Paternostro d, Elisabetta Paladino a c b, Giuseppe Falci </x:v>
+        <x:v>Yi-Pei Liu *, Qing-Shan Jia *, Xu Wang </x:v>
       </x:c>
       <x:c r="E112" t="str">
-        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0375960122001360</x:v>
+        <x:v>https://www.sciencedirect.com/science/article/pii/S2405896322011508#aep-article-footnote-id1</x:v>
       </x:c>
       <x:c r="F112" t="str">
         <x:v>QRL</x:v>
@@ -2576,19 +2576,19 @@
     </x:row>
     <x:row r="113">
       <x:c r="A113" t="str">
-        <x:v>Performance analysis of a hybrid agent for quantum-accessible reinforcement learning</x:v>
+        <x:v>Identifying optimal cycles in quantum thermal machines with reinforcement-learning</x:v>
       </x:c>
       <x:c r="B113" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C113" t="str">
-        <x:v>New Journal of Physics</x:v>
+        <x:v>npj Quantum Information</x:v>
       </x:c>
       <x:c r="D113" t="str">
-        <x:v>Arne Hamann3,1 and Sabine Wölk</x:v>
+        <x:v>Paolo A. Erdman &amp; Frank Noé </x:v>
       </x:c>
       <x:c r="E113" t="str">
-        <x:v>https://iopscience.iop.org/article/10.1088/1367-2630/ac5b56/meta</x:v>
+        <x:v>https://www.nature.com/articles/s41534-021-00512-0</x:v>
       </x:c>
       <x:c r="F113" t="str">
         <x:v>QRL</x:v>
@@ -2596,19 +2596,19 @@
     </x:row>
     <x:row r="114">
       <x:c r="A114" t="str">
-        <x:v>Deep Reinforcement Learning With Reward Design for Quantum Control</x:v>
+        <x:v>Quantum Policy Iteration via Amplitude Estimation and Grover Search -- Towards Quantum Advantage for Reinforcement Learning</x:v>
       </x:c>
       <x:c r="B114" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C114" t="str">
-        <x:v>IEEE Transactions</x:v>
+        <x:v>arxiv</x:v>
       </x:c>
       <x:c r="D114" t="str">
-        <x:v>Haixu Yu; Xudong Zhao</x:v>
+        <x:v>Simon Wiedemann, Daniel Hein, Steffen Udluft, Christian Mendl</x:v>
       </x:c>
       <x:c r="E114" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9964411</x:v>
+        <x:v>https://arxiv.org/abs/2206.04741</x:v>
       </x:c>
       <x:c r="F114" t="str">
         <x:v>QRL</x:v>
@@ -2616,19 +2616,19 @@
     </x:row>
     <x:row r="115">
       <x:c r="A115" t="str">
-        <x:v>Reinforcement-learning generation of four-qubit entangled states</x:v>
+        <x:v>Quantum Reinforcement Learning for Solving a Stochastic Frozen Lake Environment and the Impact of Quantum Architecture Choices</x:v>
       </x:c>
       <x:c r="B115" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C115" t="str">
-        <x:v>Phys. Rev. Research 4</x:v>
+        <x:v>arxiv</x:v>
       </x:c>
       <x:c r="D115" t="str">
-        <x:v>Sara Giordano and Miguel A. Martin-Delgado</x:v>
+        <x:v>Theodora-Augustina Drăgan, Maureen Monnet, Christian B. Mendl, Jeanette Miriam Lorenz</x:v>
       </x:c>
       <x:c r="E115" t="str">
-        <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.4.043056</x:v>
+        <x:v>https://arxiv.org/abs/2212.07932</x:v>
       </x:c>
       <x:c r="F115" t="str">
         <x:v>QRL</x:v>
@@ -2636,19 +2636,19 @@
     </x:row>
     <x:row r="116">
       <x:c r="A116" t="str">
-        <x:v>Quantum Reinforcement Learning—Connecting Reinforcement Learning and Quantum Computing</x:v>
+        <x:v>Quantum Multi-Agent Reinforcement Learning via Variational Quantum Circuit Design</x:v>
       </x:c>
       <x:c r="B116" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>Reinforcement Learning with Hybrid Quantum Approximation in the NISQ Context</x:v>
+        <x:v>2022 IEEE 42nd International Conference on Distributed Computing Systems (ICDCS)</x:v>
       </x:c>
       <x:c r="D116" t="str">
-        <x:v>Leonhard Kunczik</x:v>
+        <x:v>Won Joon Yun; Yunseok Kwak; Jae Pyoung Kim; Hyunhee Cho; Soyi Jung; Jihong Park</x:v>
       </x:c>
       <x:c r="E116" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-658-37616-1_4</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9912289</x:v>
       </x:c>
       <x:c r="F116" t="str">
         <x:v>QRL</x:v>
@@ -2656,19 +2656,19 @@
     </x:row>
     <x:row r="117">
       <x:c r="A117" t="str">
-        <x:v>Short quantum circuits in reinforcement learning policies for the vehicle routing problem</x:v>
+        <x:v>Efficient and robust entanglement generation with deep reinforcement learning for quantum metrology</x:v>
       </x:c>
       <x:c r="B117" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>Phys. Rev. A 105</x:v>
+        <x:v>New Journal of Physics (NJP)</x:v>
       </x:c>
       <x:c r="D117" t="str">
-        <x:v>Fabio Sanches, Sean Weinberg, Takanori Ide, and Kazumitsu Kamiya</x:v>
+        <x:v>Yuxiang Qiu, Min Zhuang, Jiahao Huang and Chaohong Lee</x:v>
       </x:c>
       <x:c r="E117" t="str">
-        <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.105.062403</x:v>
+        <x:v>https://iopscience.iop.org/article/10.1088/1367-2630/ac8285/meta</x:v>
       </x:c>
       <x:c r="F117" t="str">
         <x:v>QRL</x:v>
@@ -2676,49 +2676,209 @@
     </x:row>
     <x:row r="118">
       <x:c r="A118" t="str">
-        <x:v>A Multiagent Quantum Deep Reinforcement Learning Method for Distributed Frequency Control of Islanded Microgrids</x:v>
+        <x:v>NFT-Based Intelligence Networking for Connected and Autonomous Vehicles: A Quantum Reinforcement Learning Approach</x:v>
       </x:c>
       <x:c r="B118" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C118" t="str">
+        <x:v>IEEE Network</x:v>
+      </x:c>
+      <x:c r="D118" t="str">
+        <x:v>Yuzheng Ren; Renchao Xie; F. Richard Yu; Tao Huang; Yunjie Liu</x:v>
+      </x:c>
+      <x:c r="E118" t="str">
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9852376</x:v>
+      </x:c>
+      <x:c r="F118" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="119">
+      <x:c r="A119" t="str">
+        <x:v>Quantum imaginary time evolution steered by reinforcement learning</x:v>
+      </x:c>
+      <x:c r="B119" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C119" t="str">
+        <x:v>Communications Physics volume</x:v>
+      </x:c>
+      <x:c r="D119" t="str">
+        <x:v>      Chenfeng Cao, Zheng An, Shi-Yao Hou, D. L. Zhou &amp; Bei Zeng   </x:v>
+      </x:c>
+      <x:c r="E119" t="str">
+        <x:v>https://www.nature.com/articles/s42005-022-00837-y</x:v>
+      </x:c>
+      <x:c r="F119" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="120">
+      <x:c r="A120" t="str">
+        <x:v>A tutorial on optimal control and reinforcement learning methods for quantum technologies</x:v>
+      </x:c>
+      <x:c r="B120" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C120" t="str">
+        <x:v>Physics Letters A</x:v>
+      </x:c>
+      <x:c r="D120" t="str">
+        <x:v>Luigi Giannelli a b, Sofia Sgroi d, Jonathon Brown d, Gheorghe Sorin Paraoanu e, Mauro Paternostro d, Elisabetta Paladino a c b, Giuseppe Falci </x:v>
+      </x:c>
+      <x:c r="E120" t="str">
+        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0375960122001360</x:v>
+      </x:c>
+      <x:c r="F120" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="121">
+      <x:c r="A121" t="str">
+        <x:v>Performance analysis of a hybrid agent for quantum-accessible reinforcement learning</x:v>
+      </x:c>
+      <x:c r="B121" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C121" t="str">
+        <x:v>New Journal of Physics</x:v>
+      </x:c>
+      <x:c r="D121" t="str">
+        <x:v>Arne Hamann3,1 and Sabine Wölk</x:v>
+      </x:c>
+      <x:c r="E121" t="str">
+        <x:v>https://iopscience.iop.org/article/10.1088/1367-2630/ac5b56/meta</x:v>
+      </x:c>
+      <x:c r="F121" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="122">
+      <x:c r="A122" t="str">
+        <x:v>Deep Reinforcement Learning With Reward Design for Quantum Control</x:v>
+      </x:c>
+      <x:c r="B122" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C122" t="str">
+        <x:v>IEEE Transactions</x:v>
+      </x:c>
+      <x:c r="D122" t="str">
+        <x:v>Haixu Yu; Xudong Zhao</x:v>
+      </x:c>
+      <x:c r="E122" t="str">
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9964411</x:v>
+      </x:c>
+      <x:c r="F122" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="123">
+      <x:c r="A123" t="str">
+        <x:v>Reinforcement-learning generation of four-qubit entangled states</x:v>
+      </x:c>
+      <x:c r="B123" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C123" t="str">
+        <x:v>Phys. Rev. Research 4</x:v>
+      </x:c>
+      <x:c r="D123" t="str">
+        <x:v>Sara Giordano and Miguel A. Martin-Delgado</x:v>
+      </x:c>
+      <x:c r="E123" t="str">
+        <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.4.043056</x:v>
+      </x:c>
+      <x:c r="F123" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="124">
+      <x:c r="A124" t="str">
+        <x:v>Quantum Reinforcement Learning—Connecting Reinforcement Learning and Quantum Computing</x:v>
+      </x:c>
+      <x:c r="B124" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C124" t="str">
+        <x:v>Reinforcement Learning with Hybrid Quantum Approximation in the NISQ Context</x:v>
+      </x:c>
+      <x:c r="D124" t="str">
+        <x:v>Leonhard Kunczik</x:v>
+      </x:c>
+      <x:c r="E124" t="str">
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-658-37616-1_4</x:v>
+      </x:c>
+      <x:c r="F124" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="125">
+      <x:c r="A125" t="str">
+        <x:v>Short quantum circuits in reinforcement learning policies for the vehicle routing problem</x:v>
+      </x:c>
+      <x:c r="B125" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C125" t="str">
+        <x:v>Phys. Rev. A 105</x:v>
+      </x:c>
+      <x:c r="D125" t="str">
+        <x:v>Fabio Sanches, Sean Weinberg, Takanori Ide, and Kazumitsu Kamiya</x:v>
+      </x:c>
+      <x:c r="E125" t="str">
+        <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.105.062403</x:v>
+      </x:c>
+      <x:c r="F125" t="str">
+        <x:v>QRL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="126">
+      <x:c r="A126" t="str">
+        <x:v>A Multiagent Quantum Deep Reinforcement Learning Method for Distributed Frequency Control of Islanded Microgrids</x:v>
+      </x:c>
+      <x:c r="B126" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C126" t="str">
         <x:v>IEEE Transactions on Control of Network Systems</x:v>
       </x:c>
-      <x:c r="D118" t="str">
+      <x:c r="D126" t="str">
         <x:v>Rudai Yan; Yu Wang; Yan Xu; Jiahong Dai</x:v>
       </x:c>
-      <x:c r="E118" t="str">
+      <x:c r="E126" t="str">
         <x:v>https://ieeexplore.ieee.org/abstract/document/9670708</x:v>
       </x:c>
-      <x:c r="F118" t="str">
+      <x:c r="F126" t="str">
         <x:v>QRL</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="Rc95b8809c9394331"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="Rbda80db8934346b5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="R33b7ae0cf4c84ef7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="R9c1d0eb4cd1a42b4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="Rdfd120a5f90b4021"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="R4005a47e078d4b1f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="R478b3189103742f9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="Rd221c6d574cf4cf7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="Rb0abe162c7ec4746"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="R5e2c0155745143db"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="Rabd047256e6f4cbe"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="R1b88891454154e4c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="R2a8294adfc8e4179"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="Rebf37839a13243f5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="Rc7a43d6ef92a49a6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="Rb9ee00a50f404209"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="R0bacf0e0690c4c9d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="R1febd7e64376432f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="R261fc9d8afa24abf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="Raeb834d61ccf47ea"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="R3ec3550983764005"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="Rb67f12b724f94069"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="Rfeed6441187b43f0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="R41efc81388c1421f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="R62a7d74305dd4f60"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="R7c722f13d9fd4ab4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="Ra330a1e0b2ff4611"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="R8146f1099d984ca0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="Rd354f5ac942d461f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="R7200c8e23fe04571"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="Ra49e282b13724474"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="R0189757debec42d5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="R4f962fd5e7454719"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="R1455b1708a7a4bd9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="Racd2924c754c4462"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E73" r:id="Rb36f4c58cf6d4e6b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E74" r:id="Rb446025b6ef24cff"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E75" r:id="Rbc6890a7f1714943"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E76" r:id="Re3bc3ba2d2ba494f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="R78bc87b7b61346d8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="Rfddccc028306492a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="R2889e6343f1a40fa"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="R7418bff6a2a34d30"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E81" r:id="R97d03868384d4fdb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E82" r:id="R257007f0d9e64909"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="Rf908cc00672c4a58"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>